<commit_message>
Fix: wrong current-password attempt was force-logging users out
The change-password endpoint legitimately returns 401 for "current
password is incorrect," but the global axios interceptor treated any
401 as session-expired and nuked the whole session/redirected to
login - so a simple typo in your current password logged you out
entirely instead of showing the inline error the form already
handles. Excludes change-password from that treatment, same as
login/register already are.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/prospecting/01_Client_Gap_Matrix.xlsx
+++ b/prospecting/01_Client_Gap_Matrix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bce441479ebfac8e/Desktop/ArthaInvest/prospecting/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artha\OneDrive\Desktop\ArthaInvest\prospecting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8E1E35C-9DA0-458B-B676-E4355C6851DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B2E6A9D6-140A-4B4A-A1FC-85880DBB7B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7270" xr2:uid="{095D4074-ED0B-4F59-B75C-119BD09856CD}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7270" xr2:uid="{9F6560BB-A750-41D1-8FB9-474B900A7A8B}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -1119,7 +1119,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8285AF20-35AB-46F1-A551-24A7FF294742}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A503F6E-9174-4F93-9760-B7D9E1CE33E4}">
   <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1137,7 +1137,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>46255.390277777777</v>
+        <v>46268.388194444444</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -1265,7 +1265,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E569119-EB1E-4614-85F7-E2D5C9665CA6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D103B6F6-BF36-48EC-9023-71320FD93068}">
   <dimension ref="A1:AD28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3331,13 +3331,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD1" xr:uid="{4E569119-EB1E-4614-85F7-E2D5C9665CA6}"/>
+  <autoFilter ref="A1:AD1" xr:uid="{D103B6F6-BF36-48EC-9023-71320FD93068}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A97AD4F-B0AD-439D-AE40-22D8757526C5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E116E1F6-620D-4ACB-99F5-E7A3EDB8A49E}">
   <dimension ref="A1:M26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -4197,13 +4197,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M1" xr:uid="{6A97AD4F-B0AD-439D-AE40-22D8757526C5}"/>
+  <autoFilter ref="A1:M1" xr:uid="{E116E1F6-620D-4ACB-99F5-E7A3EDB8A49E}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C23950F-8732-4208-9645-1340CA5C9FCC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C2F9D6A-5118-4085-B85E-EED0AFCCAFCB}">
   <dimension ref="A1:N28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -4558,7 +4558,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1" xr:uid="{8C23950F-8732-4208-9645-1340CA5C9FCC}"/>
+  <autoFilter ref="A1:N1" xr:uid="{8C2F9D6A-5118-4085-B85E-EED0AFCCAFCB}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add real per-contact document storage, replacing the non-functional DigiLocker mockup
The old DigiLocker modal was UI-only from an earlier build phase - hardcoded
checkboxes, buttons with no click handlers, no backend endpoint at all.
Replaces it with a real contact_documents table, upload/list/delete
endpoints, and a working frontend panel. Uses the same S3-or-local-disk
storage convention already built for voice notes.

Also includes routine prospecting spreadsheet/dashboard updates.
</commit_message>
<xml_diff>
--- a/prospecting/01_Client_Gap_Matrix.xlsx
+++ b/prospecting/01_Client_Gap_Matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artha\OneDrive\Desktop\ArthaInvest\prospecting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B2E6A9D6-140A-4B4A-A1FC-85880DBB7B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E9B633F-16ED-45D1-A88C-4822EF3D5886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7270" xr2:uid="{9F6560BB-A750-41D1-8FB9-474B900A7A8B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1391C900-75D0-415E-A73A-CFA52DAAD5EB}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -1119,7 +1119,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A503F6E-9174-4F93-9760-B7D9E1CE33E4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C3AD8E4-F582-4401-AC2F-20F3134876C1}">
   <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1137,7 +1137,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>46268.388194444444</v>
+        <v>46270.703472222223</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -1265,7 +1265,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D103B6F6-BF36-48EC-9023-71320FD93068}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48DAC580-78AC-4659-AD73-6B948C8E42D2}">
   <dimension ref="A1:AD28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3331,13 +3331,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD1" xr:uid="{D103B6F6-BF36-48EC-9023-71320FD93068}"/>
+  <autoFilter ref="A1:AD1" xr:uid="{48DAC580-78AC-4659-AD73-6B948C8E42D2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E116E1F6-620D-4ACB-99F5-E7A3EDB8A49E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31935E05-0E57-40C5-99DB-174F011B28DD}">
   <dimension ref="A1:M26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -4197,13 +4197,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M1" xr:uid="{E116E1F6-620D-4ACB-99F5-E7A3EDB8A49E}"/>
+  <autoFilter ref="A1:M1" xr:uid="{31935E05-0E57-40C5-99DB-174F011B28DD}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C2F9D6A-5118-4085-B85E-EED0AFCCAFCB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60DD31C8-41F9-4E87-89EC-E4FAA19D7D6E}">
   <dimension ref="A1:N28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -4558,7 +4558,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1" xr:uid="{8C2F9D6A-5118-4085-B85E-EED0AFCCAFCB}"/>
+  <autoFilter ref="A1:N1" xr:uid="{60DD31C8-41F9-4E87-89EC-E4FAA19D7D6E}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>